<commit_message>
⏱ All Timeframe scan [2026-08-31]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -33272,7 +33272,7 @@
       </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t>151235.04 - 159415.43 RD SUPPLY</t>
+          <t>151235.03 - 159415.43 RD SUPPLY</t>
         </is>
       </c>
       <c r="I314" t="inlineStr">
@@ -33374,7 +33374,7 @@
       </c>
       <c r="H315" t="inlineStr">
         <is>
-          <t>10163.48 - 12763.22 DR DEMAND</t>
+          <t>10163.49 - 12763.22 DR DEMAND</t>
         </is>
       </c>
       <c r="I315" t="inlineStr">
@@ -36522,11 +36522,11 @@
         </is>
       </c>
       <c r="E346" t="n">
-        <v>2515</v>
+        <v>2512.5</v>
       </c>
       <c r="F346" t="inlineStr">
         <is>
-          <t>2252.1 - 2342.0 DR DEMAND</t>
+          <t>2249.86 - 2339.67 DR DEMAND</t>
         </is>
       </c>
       <c r="G346" t="inlineStr">
@@ -36536,7 +36536,7 @@
       </c>
       <c r="H346" t="inlineStr">
         <is>
-          <t>1274.17 - 1542.62 DR DEMAND</t>
+          <t>1272.91 - 1541.08 DR DEMAND</t>
         </is>
       </c>
       <c r="I346" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-09-01]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -13894,7 +13894,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>10163.49 - 12763.22 DR DEMAND</t>
+          <t>10163.48 - 12763.22 DR DEMAND</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -35292,7 +35292,7 @@
       </c>
       <c r="H334" t="inlineStr">
         <is>
-          <t>1598.44 - 1928.41 RD SUPPLY</t>
+          <t>1598.43 - 1928.41 RD SUPPLY</t>
         </is>
       </c>
       <c r="I334" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-09-02]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -13588,7 +13588,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>10163.49 - 12763.22 DR DEMAND</t>
+          <t>10163.48 - 12763.22 DR DEMAND</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -34036,7 +34036,7 @@
       </c>
       <c r="H322" t="inlineStr">
         <is>
-          <t>1598.43 - 1928.41 RD SUPPLY</t>
+          <t>1598.44 - 1928.41 RD SUPPLY</t>
         </is>
       </c>
       <c r="I322" t="inlineStr">
@@ -38218,7 +38218,7 @@
       </c>
       <c r="H363" t="inlineStr">
         <is>
-          <t>550.35 - 680.06 DR DEMAND</t>
+          <t>550.35 - 680.07 DR DEMAND</t>
         </is>
       </c>
       <c r="I363" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-09-03]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -13926,7 +13926,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>10163.49 - 12763.22 DR DEMAND</t>
+          <t>10163.48 - 12763.22 DR DEMAND</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -31408,7 +31408,7 @@
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>4334.99 - 4897.45 RD SUPPLY</t>
+          <t>4335.0 - 4897.45 RD SUPPLY</t>
         </is>
       </c>
       <c r="I296" t="inlineStr">
@@ -36406,7 +36406,7 @@
       </c>
       <c r="H345" t="inlineStr">
         <is>
-          <t>1598.43 - 1928.41 RD SUPPLY</t>
+          <t>1598.44 - 1928.41 RD SUPPLY</t>
         </is>
       </c>
       <c r="I345" t="inlineStr">
@@ -40384,7 +40384,7 @@
       </c>
       <c r="H384" t="inlineStr">
         <is>
-          <t>550.35 - 680.07 DR DEMAND</t>
+          <t>550.35 - 680.06 DR DEMAND</t>
         </is>
       </c>
       <c r="I384" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-09-08]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -918,7 +918,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>10163.48 - 12763.22 DR DEMAND</t>
+          <t>10163.49 - 12763.22 DR DEMAND</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>101787.0 - 115617.15 DR DEMAND</t>
+          <t>101786.99 - 115617.15 DR DEMAND</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -31172,7 +31172,7 @@
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>1598.43 - 1928.41 RD SUPPLY</t>
+          <t>1598.44 - 1928.41 RD SUPPLY</t>
         </is>
       </c>
       <c r="I294" t="inlineStr">
@@ -39230,7 +39230,7 @@
       </c>
       <c r="H373" t="inlineStr">
         <is>
-          <t>550.35 - 680.07 DR DEMAND</t>
+          <t>550.35 - 680.06 DR DEMAND</t>
         </is>
       </c>
       <c r="I373" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-09-09]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -698,7 +698,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>10163.49 - 12763.22 DR DEMAND</t>
+          <t>10163.48 - 12763.22 DR DEMAND</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -30858,7 +30858,7 @@
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>4335.0 - 4897.45 RD SUPPLY</t>
+          <t>4334.99 - 4897.45 RD SUPPLY</t>
         </is>
       </c>
       <c r="I291" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-09-10]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -31940,7 +31940,7 @@
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t>4334.99 - 4897.45 RD SUPPLY</t>
+          <t>4335.0 - 4897.45 RD SUPPLY</t>
         </is>
       </c>
       <c r="I302" t="inlineStr">
@@ -32348,7 +32348,7 @@
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>1598.43 - 1928.41 RD SUPPLY</t>
+          <t>1598.44 - 1928.41 RD SUPPLY</t>
         </is>
       </c>
       <c r="I306" t="inlineStr">
@@ -39394,7 +39394,7 @@
       </c>
       <c r="H375" t="inlineStr">
         <is>
-          <t>550.35 - 680.06 DR DEMAND</t>
+          <t>550.35 - 680.07 DR DEMAND</t>
         </is>
       </c>
       <c r="I375" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-09-11]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -9050,7 +9050,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>10163.48 - 12763.22 DR DEMAND</t>
+          <t>10163.49 - 12763.22 DR DEMAND</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -37910,7 +37910,7 @@
       </c>
       <c r="H361" t="inlineStr">
         <is>
-          <t>550.35 - 680.06 DR DEMAND</t>
+          <t>550.35 - 680.07 DR DEMAND</t>
         </is>
       </c>
       <c r="I361" t="inlineStr">

</xml_diff>